<commit_message>
upgrade: update snapshot 20260901;
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -1,26 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alef.xu/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F432A571-0EF3-E04D-865C-FA4BF3D9F91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B3747A0-AE08-B541-99F3-9E44A24EFA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="500" windowWidth="28100" windowHeight="16460" xr2:uid="{4A9CE4A5-B555-5344-96E6-FBE81B63CA5B}"/>
+    <workbookView xWindow="3220" yWindow="2140" windowWidth="28100" windowHeight="17360" xr2:uid="{03C76504-C1EF-8B4F-A950-9E551D24283C}"/>
   </bookViews>
   <sheets>
-    <sheet name="huobi_por (1)" sheetId="1" r:id="rId1"/>
+    <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="137">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="265" uniqueCount="98">
   <si>
     <t>coin</t>
   </si>
@@ -67,27 +72,15 @@
     <t>stETH</t>
   </si>
   <si>
-    <t>ETH</t>
-  </si>
-  <si>
-    <t>ETH-ARB</t>
-  </si>
-  <si>
     <t>HTX(All)</t>
   </si>
   <si>
-    <t>232059560281012.00</t>
-  </si>
-  <si>
     <t>HTX-ERC20</t>
   </si>
   <si>
     <t>HTX-TRC20</t>
   </si>
   <si>
-    <t>231371738784003.00</t>
-  </si>
-  <si>
     <t>SOL(All)</t>
   </si>
   <si>
@@ -124,9 +117,6 @@
     <t>USDT(All)</t>
   </si>
   <si>
-    <t>USDT-ERC20</t>
-  </si>
-  <si>
     <t>USDT-TRC20</t>
   </si>
   <si>
@@ -145,9 +135,6 @@
     <t>TRC20-USDD</t>
   </si>
   <si>
-    <t>USDD-BEP20</t>
-  </si>
-  <si>
     <t>jUSDD-TRC20</t>
   </si>
   <si>
@@ -220,6 +207,9 @@
     <t>TK86Qm97uM848dMk8G7xNbJB7zG1uW3h1n</t>
   </si>
   <si>
+    <t>DQhEuTa5UkNcD8YFZK3pvjFfrtMqQpJhSa</t>
+  </si>
+  <si>
     <t>DRRU8L7fF4k9w7SF3Z6ei8onPCsh9hjGX1</t>
   </si>
   <si>
@@ -250,99 +240,24 @@
     <t>DB5KWytcxHyphHPn9iC92Y9JqPRL1Fq21p</t>
   </si>
   <si>
-    <t>DArSwetSeoQSWuCkqTCGrPd8BYa5EfUBMW</t>
-  </si>
-  <si>
-    <t>9ztZpRN3v9xv5JhAT7MTtmy4DfyMEAG8YU</t>
-  </si>
-  <si>
-    <t>DJX3kCZfcDuREturnUNKEBQELi1PFaLkJC</t>
-  </si>
-  <si>
-    <t>DKs2WBbiaAEe9RGzQTmtJj1o9bqsKTUTtC</t>
-  </si>
-  <si>
-    <t>A8GUArLTCASQAtcqLT6w8U3vyGm3qipf1h</t>
-  </si>
-  <si>
-    <t>9w9HgRZwA9LFTSALD7tK6qkcrhyzBRuFrT</t>
-  </si>
-  <si>
     <t>DP9QNiRnJ1anxwC8LvNPLS1QQc2YoTHd4D</t>
   </si>
   <si>
+    <t>D8fLX1YZnMNnDbwi8NbPZ3m3ZUYSHx4DkF</t>
+  </si>
+  <si>
+    <t>ADwSjbA8Edsk6GHubJnp8vEu9fqHV4PvJ3</t>
+  </si>
+  <si>
     <t>0x6663613fbd927ce78abbf7f5ca7e2c3fe0d96d18</t>
   </si>
   <si>
-    <t>0x4fb312915b779b1339388e14b6d079741ca83128</t>
-  </si>
-  <si>
-    <t>0xef72CC0Bb3EE2236b3B875C66a8A5D06b53Adb99</t>
-  </si>
-  <si>
-    <t>htx</t>
-  </si>
-  <si>
-    <t>0xc91377206d5903eff7c725d0ab54ed1a652110581e449c5ccc7f4f5bb991af80228ae4a95f448bb18a6ac78e850334daa495930b85375f3d6ab606ac0146d8b61b</t>
-  </si>
-  <si>
-    <t>0x406ea8F3C6464171f3dEccF6Ba99748D9487CD52</t>
-  </si>
-  <si>
-    <t>0x3ba1542404430b5818a403ab451e4ee2299a0b9e8c2d71f178edf0e2c4df222a77ac3dd16011369cc395063da048e975620ddc6e511f762ad639640ca8d4fac31c</t>
-  </si>
-  <si>
-    <t>0x3f95d25BfB08e6cF5bA3e159e477D28852BA3F04</t>
-  </si>
-  <si>
-    <t>0xc766bb36b671096e668bd902515eecef9939bcd99226bb668768f7d3a2cc5387339c98d0d8f21a3f3ec27024ccfeb5034d617a4d6021cab5538f061f198808d31b</t>
-  </si>
-  <si>
-    <t>0x9EC19cE75a7557d52c32774779158F5A466e0080</t>
-  </si>
-  <si>
-    <t>0x0d929c70239b715b65f891088a5143e21449c36cab4243f71e5ce84317454c6605013fad579dc198c43798e2a9e7d575a9c39fc67689a2b4e38635e2e934ef661c</t>
-  </si>
-  <si>
-    <t>0x9be5b8a7314552fa47feb1355cd5b4adc7bb7516</t>
-  </si>
-  <si>
-    <t>0xa49abf338f924c7ba547a37a56ad5c22947451fc1171d954ea0793376adfd80d370742f5cdff9e1fd24bf3ba157421854b3e7d80e17d8ad181c56321eadb50641c</t>
-  </si>
-  <si>
-    <t>0x68ad2e694c6be593f5b7dda2e8f1a8915b735331</t>
-  </si>
-  <si>
-    <t>0xa2fdd96d04abfe1721944a9ef7b41b8ce54060ea29bc49fc87710ff59f5bcc9556f9ef323ea85e7cbe00f71770757e3625c15ffa34a39c47f79a9a95cc88b8cb1c</t>
-  </si>
-  <si>
-    <t>0x1c1b34a6ba2b81d3ce5bd3c35a29da0cbab42c56</t>
-  </si>
-  <si>
-    <t>0xc72caa65282c9bbeac036897b7cc120fc76f498b7bcda6abfe7533fb9b09578f7cd4d4e9ed91fe42f74a419c20ff6947950114bf2254a4058fd4452a543f316a1b</t>
-  </si>
-  <si>
-    <t>0x2f313a0bd2f885ddc4a3d990d4effccfc659c202</t>
-  </si>
-  <si>
-    <t>0x1185e3ccf6f582a0fa720214be009a7165096d0d3bbbca14abdf5e3fba411cde5860691c78b922090911fbf1540bd2f75b0ad90a22c1a0db4c46b9cbbfdf0a061b</t>
-  </si>
-  <si>
-    <t>0x82d015d74670d8645b56c3f453398a3e799ee582</t>
-  </si>
-  <si>
     <t>0x18709e89bd403f470088abdacebe86cc60dda12e</t>
   </si>
   <si>
     <t>0x68a79a40adfb16777e49206d60f9cd11de0fbaf3acad5be1e30dd955182475f43255dfec5fede4dc97fcf1fbce1583dd05ee419bf3939ca95919aff931eec41d01</t>
   </si>
   <si>
-    <t>230974428784003.00</t>
-  </si>
-  <si>
-    <t>5bJcc9eb2XE7mqcET2xDuAdMGuXWybb4YPmAHLjKLhQG</t>
-  </si>
-  <si>
     <t>TYh6mgoMNZTCsgpYHBz7gttEfrQmDMABub</t>
   </si>
   <si>
@@ -391,34 +306,7 @@
     <t>51fbb14497b6f5265b44931dac48e23822b645598d7a9c5fee183c9a517db9491594b82a03e1dfea9072e3e95a29d5716610f5aefdbd934fab8b67d73f148d6900</t>
   </si>
   <si>
-    <t>0xafdfd157d9361e621e476036fee62f688450692b</t>
-  </si>
-  <si>
-    <t>USDT-ETH</t>
-  </si>
-  <si>
-    <t>0x2a4bf9bbca7a91661087f52571eea36a004b83eb</t>
-  </si>
-  <si>
-    <t>0x9e2b154db03c9cf389c2ff9f3921299f2ec7fb4893b91893855a7e2627783a7159f2e798c0450013d11961db1f100fc8a59dbd49384a1cbae160820f6165457c1c</t>
-  </si>
-  <si>
-    <t>TWN6yGR6VzYmThSy2CmkpEASyvwV4VKRDs</t>
-  </si>
-  <si>
-    <t>0x4c1d4b5922317f58967c3759c6bbeb57497e40e81662260ae8fa82496d0c391467a0d0cf7d8bd9039594057c4353c7d7831c247912148a62f9548282372a551700</t>
-  </si>
-  <si>
-    <t>TB5s4duG2LqfnkF1VgX4fWdvtYcmf1WELk</t>
-  </si>
-  <si>
-    <t>0xf0d92874a3a44f7ecaec706de6c481f003baab5373c0cd98c73aa2d911ff029a432e8c42150546d1a72b21cf0326a28077fa01e4c6d91a256b13c225c84b26b901</t>
-  </si>
-  <si>
-    <t>THBF3NdL2qRJc19eDCrC5atW3Tdkcg4oMB</t>
-  </si>
-  <si>
-    <t>0x3ca7a1fcc5306107b4bd37c82359ec2a1c62b32658bb01201f12bf5e9e1b5c54623f440d226165bf4d216cffe5a4e3fce9e636e7514eac5c29af97df12e88fd400</t>
+    <t>0xdaa4393013f359fd63a133a3b893d311aba4e471</t>
   </si>
   <si>
     <t>TBuzWQynfzershAsPfGjo4A9sXUfZf8wsq</t>
@@ -436,9 +324,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.00_ "/>
+    <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -784,15 +672,15 @@
   </fills>
   <borders count="11">
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4"/>
@@ -800,8 +688,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4" tint="0.499984740745262"/>
@@ -809,8 +697,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.39997558519241921"/>
@@ -818,12 +706,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FF7F7F7F"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FF7F7F7F"/>
       </top>
@@ -833,12 +721,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FF3F3F3F"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -848,8 +736,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
@@ -857,12 +745,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
+      <start style="double">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
+      </start>
+      <end style="double">
         <color rgb="FF3F3F3F"/>
-      </right>
+      </end>
       <top style="double">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -872,12 +760,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FFB2B2B2"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FFB2B2B2"/>
       </top>
@@ -887,8 +775,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -898,12 +786,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color indexed="64"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color indexed="64"/>
-      </right>
+      </end>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -1041,20 +929,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1116,7 +998,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://purl.oclc.org/ooxml/drawingml/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1269,25 +1151,25 @@
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:lumMod val="110%"/>
+                <a:satMod val="105%"/>
+                <a:tint val="67%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="103%"/>
+                <a:tint val="73%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="109%"/>
+                <a:tint val="81%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1295,25 +1177,25 @@
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:satMod val="103%"/>
+                <a:lumMod val="102%"/>
+                <a:tint val="94%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:satMod val="110%"/>
+                <a:lumMod val="100%"/>
+                <a:shade val="100%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:lumMod val="99%"/>
+                <a:satMod val="120%"/>
+                <a:shade val="78%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1326,21 +1208,21 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1354,7 +1236,7 @@
           <a:effectLst>
             <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="63%"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -1366,32 +1248,32 @@
         </a:solidFill>
         <a:solidFill>
           <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
+            <a:tint val="95%"/>
+            <a:satMod val="170%"/>
           </a:schemeClr>
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="93%"/>
+                <a:satMod val="150%"/>
+                <a:shade val="98%"/>
+                <a:lumMod val="102%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="98%"/>
+                <a:satMod val="130%"/>
+                <a:shade val="90%"/>
+                <a:lumMod val="103%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="63%"/>
+                <a:satMod val="120%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1431,13 +1313,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A2530E6-76DB-AC46-9A7D-F0CC8515CC8F}">
-  <dimension ref="A1:F124"/>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD334E2B-7567-3B4F-9978-76C3980BF025}">
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="41.6640625" customWidth="1"/>
-    <col min="3" max="3" width="43.83203125" customWidth="1"/>
-    <col min="6" max="6" width="98.1640625" customWidth="1"/>
+    <col min="2" max="2" width="45.33203125" customWidth="1"/>
+    <col min="3" max="3" width="49.6640625" customWidth="1"/>
+    <col min="4" max="4" width="63.5" customWidth="1"/>
+    <col min="5" max="5" width="22.1640625" customWidth="1"/>
+    <col min="6" max="6" width="127.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1459,7 +1343,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1">
-        <v>20471.89</v>
+        <v>20252.349999999999</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1467,10 +1351,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="1">
-        <v>960427</v>
+        <v>964902</v>
       </c>
       <c r="C3" s="1">
-        <v>8208.93</v>
+        <v>8083.39</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1478,10 +1362,10 @@
         <v>6</v>
       </c>
       <c r="B4" s="1">
-        <v>436386797</v>
+        <v>443191405</v>
       </c>
       <c r="C4" s="1">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1489,10 +1373,10 @@
         <v>7</v>
       </c>
       <c r="B5" s="1">
-        <v>84947615</v>
+        <v>85840149</v>
       </c>
       <c r="C5" s="1">
-        <v>10398.93</v>
+        <v>10308.93</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1500,7 +1384,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="1">
-        <v>84947615</v>
+        <v>85840149</v>
       </c>
       <c r="C6" s="1">
         <v>89</v>
@@ -1525,7 +1409,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="1">
-        <v>450816847.68000001</v>
+        <v>422760583.18000001</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1533,10 +1417,10 @@
         <v>12</v>
       </c>
       <c r="B9" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="C9" s="1">
-        <v>450816847.68000001</v>
+        <v>422760583.18000001</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1547,7 +1431,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="1">
-        <v>122626.95</v>
+        <v>116757.07</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1555,404 +1439,440 @@
         <v>14</v>
       </c>
       <c r="B11" s="1">
-        <v>25653898</v>
+        <v>25876316</v>
       </c>
       <c r="C11" s="1">
-        <v>29158.34</v>
+        <v>29213.08</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="1">
-        <v>25653898</v>
+        <v>9</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="C12" s="1">
-        <v>1504.17</v>
+        <v>87543.99</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="1">
-        <v>489687604</v>
-      </c>
-      <c r="C13" s="1">
-        <v>438.57</v>
+        <v>15</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2">
+        <v>232059560281012</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1">
-        <v>91525.87</v>
+        <v>16</v>
+      </c>
+      <c r="B14" s="1">
+        <v>25876316</v>
+      </c>
+      <c r="C14" s="2">
+        <v>386057650000</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>18</v>
+      <c r="B15" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="C15" s="2">
+        <v>231371738784003</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="C16" s="3">
-        <v>386057650000</v>
+        <v>9</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="2">
+        <v>301763847007.95001</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="1">
+        <v>401370.12</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="4">
-        <v>301763847007.95001</v>
+        <v>19</v>
+      </c>
+      <c r="B18" s="1">
+        <v>443191405</v>
+      </c>
+      <c r="C18" s="1">
+        <v>399536.39</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C19" s="1">
-        <v>424080.45</v>
+        <v>1833.73</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="1">
-        <v>436386797</v>
+        <v>20</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C20" s="1">
-        <v>422246.72</v>
+        <v>9384209885.7199993</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="B21" s="1">
+        <v>85840149</v>
       </c>
       <c r="C21" s="1">
-        <v>1833.73</v>
+        <v>8461736079.7799997</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>4</v>
+        <v>22</v>
+      </c>
+      <c r="B22" s="1">
+        <v>85840149</v>
       </c>
       <c r="C22" s="1">
-        <v>9375673533.8600006</v>
+        <v>922473805.94000006</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="1">
-        <v>84947615</v>
+        <v>23</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C23" s="1">
-        <v>8453199727.9200001</v>
+        <v>27381853.73</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B24" s="1">
-        <v>84947615</v>
+        <v>106670116</v>
       </c>
       <c r="C24" s="1">
-        <v>922473805.94000006</v>
+        <v>27381853.73</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="1">
-        <v>29018853.73</v>
+        <v>240401886.12</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B26" s="1">
-        <v>105979279</v>
+        <v>443191405</v>
       </c>
       <c r="C26" s="1">
-        <v>29018853.73</v>
+        <v>972000</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C27" s="1">
-        <v>218469322.46000001</v>
+        <v>239429886.12</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="1">
-        <v>436386797</v>
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C28" s="1">
-        <v>1041000</v>
+        <v>32904965.5</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>10</v>
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>85840149</v>
       </c>
       <c r="C29" s="1">
-        <v>217428322.46000001</v>
+        <v>14984999</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C30" s="1">
-        <v>33108901.489999998</v>
+        <v>17919966.5</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="1">
-        <v>84947615</v>
+        <v>29</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C31" s="1">
-        <v>19984999</v>
+        <v>588327863.60000002</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>10</v>
+        <v>30</v>
+      </c>
+      <c r="B32" s="1">
+        <v>85840149</v>
       </c>
       <c r="C32" s="1">
-        <v>13123902.49</v>
+        <v>1909070.4</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>4</v>
+        <v>31</v>
+      </c>
+      <c r="B33" s="1">
+        <v>85840149</v>
       </c>
       <c r="C33" s="1">
-        <v>709756398.80999994</v>
+        <v>39548690.640000001</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B34" s="1">
-        <v>25653898</v>
+        <v>9</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="C34" s="1">
-        <v>1045412.19</v>
+        <v>546870102.55999994</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" s="1">
-        <v>84947615</v>
+        <v>32</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C35" s="1">
-        <v>13239070.4</v>
+        <v>360949.9</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B36" s="1">
-        <v>84947615</v>
+        <v>25876316</v>
       </c>
       <c r="C36" s="1">
-        <v>39548690.640000001</v>
+        <v>360949.9</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C37" s="1">
-        <v>655923225.59000003</v>
+        <v>131071466.44</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>4</v>
+        <v>35</v>
+      </c>
+      <c r="B38" s="1">
+        <v>85840149</v>
       </c>
       <c r="C38" s="1">
-        <v>670002.43999999994</v>
+        <v>2681000</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B39" s="1">
-        <v>25653898</v>
+        <v>85840149</v>
       </c>
       <c r="C39" s="1">
-        <v>670002.43999999994</v>
+        <v>76466743.670000002</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>4</v>
+        <v>37</v>
+      </c>
+      <c r="B40" s="1">
+        <v>25876316</v>
       </c>
       <c r="C40" s="1">
-        <v>128395203.43000001</v>
+        <v>44975772</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B41" s="1">
-        <v>84947615</v>
+        <v>9</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="C41" s="1">
-        <v>516447.15</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B42" s="1">
-        <v>113328368</v>
-      </c>
-      <c r="C42" s="1">
-        <v>3356000</v>
+        <v>6947950.7699999996</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B43" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="C43" s="1">
-        <v>76466743.670000002</v>
+        <v>0</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C44" s="1">
+        <v>964902</v>
+      </c>
+      <c r="D44" s="1">
+        <v>6132.7</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B44" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="C44" s="1">
-        <v>44975772</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="C45" s="1">
-        <v>3080240.61</v>
+        <v>964902</v>
+      </c>
+      <c r="D45" s="1">
+        <v>970.8</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C46" s="1">
+        <v>964902</v>
+      </c>
+      <c r="D46" s="1">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>2</v>
+        <v>49</v>
+      </c>
+      <c r="C47" s="1">
+        <v>964902</v>
+      </c>
+      <c r="D47" s="1">
+        <v>829.68</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1960,19 +1880,19 @@
         <v>5</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C48" s="1">
-        <v>960427</v>
+        <v>964902</v>
       </c>
       <c r="D48" s="1">
-        <v>6132.7</v>
+        <v>80.569999999999993</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1980,19 +1900,19 @@
         <v>5</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C49" s="1">
-        <v>960427</v>
+        <v>964902</v>
       </c>
       <c r="D49" s="1">
-        <v>970.8</v>
+        <v>46.26</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2000,53 +1920,53 @@
         <v>5</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C50" s="1">
-        <v>960427</v>
+        <v>964902</v>
       </c>
       <c r="D50" s="1">
-        <v>8.3800000000000008</v>
+        <v>15</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C51" s="1">
-        <v>960427</v>
+        <v>443191405</v>
       </c>
       <c r="D51" s="1">
-        <v>829.68</v>
+        <v>65</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>56</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C52" s="1">
-        <v>960427</v>
+        <v>443191405</v>
       </c>
       <c r="D52" s="1">
-        <v>80.569999999999993</v>
+        <v>17</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>4</v>
@@ -2057,36 +1977,36 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B53" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C53" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D53" s="1">
+        <v>10298.93</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C53" s="1">
-        <v>960427</v>
-      </c>
-      <c r="D53" s="1">
-        <v>34.770000000000003</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C54" s="1">
-        <v>960427</v>
+        <v>85840149</v>
       </c>
       <c r="D54" s="1">
-        <v>152.02000000000001</v>
+        <v>10</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>4</v>
@@ -2097,36 +2017,36 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C55" s="1">
-        <v>436386797</v>
+        <v>85840149</v>
       </c>
       <c r="D55" s="1">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C56" s="1">
-        <v>436386797</v>
+        <v>6355057</v>
       </c>
       <c r="D56" s="1">
-        <v>21</v>
+        <v>1189758.8700000001</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>4</v>
@@ -2137,36 +2057,36 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C57" s="1">
-        <v>84947615</v>
+        <v>6355057</v>
       </c>
       <c r="D57" s="1">
-        <v>10313.93</v>
+        <v>342891003.5</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>64</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C58" s="1">
-        <v>84947615</v>
+        <v>6355057</v>
       </c>
       <c r="D58" s="1">
-        <v>85</v>
+        <v>66066923.390000001</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>4</v>
@@ -2177,22 +2097,22 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C59" s="1">
-        <v>84947615</v>
+        <v>6355057</v>
       </c>
       <c r="D59" s="1">
-        <v>89</v>
+        <v>2866994</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>64</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2200,13 +2120,13 @@
         <v>12</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C60" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D60" s="1">
-        <v>353891003.5</v>
+        <v>2647816.5299999998</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>4</v>
@@ -2220,13 +2140,13 @@
         <v>12</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C61" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D61" s="1">
-        <v>66066923.390000001</v>
+        <v>1457329.63</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>4</v>
@@ -2240,13 +2160,13 @@
         <v>12</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C62" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D62" s="1">
-        <v>2866994</v>
+        <v>1066964.3</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>4</v>
@@ -2260,13 +2180,13 @@
         <v>12</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C63" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D63" s="1">
-        <v>2647816.5299999998</v>
+        <v>850746.71</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>4</v>
@@ -2280,13 +2200,13 @@
         <v>12</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C64" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D64" s="1">
-        <v>1457329.63</v>
+        <v>579364.13</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>4</v>
@@ -2300,13 +2220,13 @@
         <v>12</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C65" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D65" s="1">
-        <v>1066964.3</v>
+        <v>538350.48</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>4</v>
@@ -2320,13 +2240,13 @@
         <v>12</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C66" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D66" s="1">
-        <v>850746.71</v>
+        <v>127419.44</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>4</v>
@@ -2340,13 +2260,13 @@
         <v>12</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C67" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D67" s="1">
-        <v>579364.13</v>
+        <v>999998.92</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>4</v>
@@ -2360,13 +2280,13 @@
         <v>12</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C68" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D68" s="1">
-        <v>538350.48</v>
+        <v>999999.11</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>4</v>
@@ -2380,13 +2300,13 @@
         <v>12</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C69" s="1">
-        <v>6312765</v>
+        <v>6355057</v>
       </c>
       <c r="D69" s="1">
-        <v>127419.44</v>
+        <v>477914.18</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>4</v>
@@ -2397,16 +2317,16 @@
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C70" s="1">
-        <v>6312765</v>
+        <v>25876316</v>
       </c>
       <c r="D70" s="1">
-        <v>339707.75</v>
+        <v>29213.08</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>4</v>
@@ -2417,56 +2337,56 @@
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C71" s="1">
-        <v>6312765</v>
-      </c>
-      <c r="D71" s="1">
-        <v>5908000.7599999998</v>
+        <v>25876316</v>
+      </c>
+      <c r="D71" s="2">
+        <v>386057650000</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="C72" s="1">
-        <v>6312765</v>
-      </c>
-      <c r="D72" s="1">
-        <v>1002473.25</v>
+        <v>85840149</v>
+      </c>
+      <c r="D72" s="2">
+        <v>230974428784003</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="C73" s="1">
-        <v>6312765</v>
-      </c>
-      <c r="D73" s="1">
-        <v>404835.24</v>
+        <v>85840149</v>
+      </c>
+      <c r="D73" s="2">
+        <v>397310000000</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>4</v>
@@ -2477,16 +2397,16 @@
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C74" s="1">
-        <v>6312765</v>
+        <v>443191405</v>
       </c>
       <c r="D74" s="1">
-        <v>10375920.15</v>
+        <v>399536.39</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>4</v>
@@ -2497,336 +2417,336 @@
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C75" s="1">
-        <v>6312765</v>
+        <v>85840149</v>
       </c>
       <c r="D75" s="1">
-        <v>1692999.51</v>
+        <v>1082089494.28</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>4</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C76" s="1">
-        <v>6312765</v>
+        <v>85840149</v>
       </c>
       <c r="D76" s="1">
-        <v>999998.92</v>
+        <v>1705110564.0899999</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C77" s="1">
-        <v>25653898</v>
+        <v>85840149</v>
       </c>
       <c r="D77" s="1">
-        <v>29158.34</v>
+        <v>755759959.02999997</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>4</v>
+        <v>82</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B78" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C78" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D78" s="1">
+        <v>1071286648.08</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F78" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C78" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="D78" s="1">
-        <v>135</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C79" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>4</v>
+      <c r="C79" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D79" s="1">
+        <v>1070397075.17</v>
       </c>
       <c r="E79" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F79" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B80" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C80" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D80" s="1">
+        <v>1144452002.4400001</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F80" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B81" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C81" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D81" s="1">
+        <v>1632640336.6900001</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F81" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B82" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C82" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D82" s="1">
+        <v>922473805.94000006</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F82" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="1" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="C83" s="1">
-        <v>25653898</v>
+        <v>85840149</v>
       </c>
       <c r="D83" s="1">
-        <v>256.26</v>
+        <v>14984999</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="1" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="C84" s="1">
-        <v>25653898</v>
+        <v>443191405</v>
       </c>
       <c r="D84" s="1">
-        <v>112.2</v>
+        <v>972000</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>97</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="1" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>98</v>
+        <v>59</v>
       </c>
       <c r="C85" s="1">
-        <v>25653898</v>
+        <v>85840149</v>
       </c>
       <c r="D85" s="1">
-        <v>1000.7</v>
+        <v>2681000</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>99</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="1" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="C86" s="1">
-        <v>489687604</v>
+        <v>85840149</v>
       </c>
       <c r="D86" s="1">
-        <v>186.58</v>
+        <v>76466743.670000002</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>101</v>
+        <v>58</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="1" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="C87" s="1">
-        <v>489687604</v>
+        <v>25876316</v>
       </c>
       <c r="D87" s="1">
-        <v>252</v>
+        <v>44975772</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C88" s="1">
-        <v>25653898</v>
+        <v>25876316</v>
       </c>
       <c r="D88" s="1">
-        <v>386057650000</v>
+        <v>360949.9</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>104</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="C89" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>105</v>
+        <v>85840149</v>
+      </c>
+      <c r="D89" s="1">
+        <v>1909070.4</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="1" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C90" s="1">
-        <v>84947615</v>
+        <v>85840149</v>
       </c>
       <c r="D90" s="1">
-        <v>397310000000</v>
+        <v>39548690.640000001</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C91" s="1">
-        <v>436386797</v>
+        <v>106670116</v>
       </c>
       <c r="D91" s="1">
-        <v>15800</v>
+        <v>26487852.739999998</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>4</v>
@@ -2837,667 +2757,26 @@
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="C92" s="1">
-        <v>436386797</v>
+        <v>106670116</v>
       </c>
       <c r="D92" s="1">
-        <v>406446.72</v>
+        <v>894000.99</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6">
-      <c r="A93" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C93" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D93" s="1">
-        <v>1082087681.4200001</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F93" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6">
-      <c r="A94" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C94" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D94" s="1">
-        <v>27225218.359999999</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6">
-      <c r="A95" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C95" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D95" s="1">
-        <v>1705110564.0899999</v>
-      </c>
-      <c r="E95" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F95" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6">
-      <c r="A96" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C96" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D96" s="1">
-        <v>755759959.02999997</v>
-      </c>
-      <c r="E96" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F96" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6">
-      <c r="A97" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C97" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D97" s="1">
-        <v>1071282890.67</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F97" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6">
-      <c r="A98" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B98" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C98" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D98" s="1">
-        <v>1070395130.62</v>
-      </c>
-      <c r="E98" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F98" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6">
-      <c r="A99" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C99" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D99" s="1">
-        <v>1144450189.5799999</v>
-      </c>
-      <c r="E99" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F99" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6">
-      <c r="A100" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C100" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D100" s="1">
-        <v>1596888094.1600001</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6">
-      <c r="A101" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C101" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D101" s="1">
-        <v>922473805.94000006</v>
-      </c>
-      <c r="E101" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F101" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6">
-      <c r="A102" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C102" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D102" s="1">
-        <v>19984999</v>
-      </c>
-      <c r="E102" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F102" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6">
-      <c r="A103" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C103" s="1">
-        <v>436386797</v>
-      </c>
-      <c r="D103" s="1">
-        <v>1041000</v>
-      </c>
-      <c r="E103" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F103" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6">
-      <c r="A104" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C104" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D104" s="1">
-        <v>297692.15000000002</v>
-      </c>
-      <c r="E104" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F104" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6">
-      <c r="A105" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C105" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D105" s="1">
-        <v>218755</v>
-      </c>
-      <c r="E105" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F105" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6">
-      <c r="A106" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C106" s="1">
-        <v>113328368</v>
-      </c>
-      <c r="D106" s="1">
-        <v>1543000</v>
-      </c>
-      <c r="E106" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F106" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6">
-      <c r="A107" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C107" s="1">
-        <v>113328368</v>
-      </c>
-      <c r="D107" s="1">
-        <v>1813000</v>
-      </c>
-      <c r="E107" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F107" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6">
-      <c r="A108" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B108" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C108" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D108" s="1">
-        <v>76466743.670000002</v>
-      </c>
-      <c r="E108" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F108" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6">
-      <c r="A109" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B109" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C109" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="D109" s="1">
-        <v>44975772</v>
-      </c>
-      <c r="E109" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F109" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6">
-      <c r="A110" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B110" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C110" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="D110" s="1">
-        <v>473679.11</v>
-      </c>
-      <c r="E110" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F110" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6">
-      <c r="A111" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B111" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D111" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E111" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F111" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6">
-      <c r="A112" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B112" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C112" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D112" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E112" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F112" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6">
-      <c r="A113" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B113" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D113" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E113" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F113" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6">
-      <c r="A114" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B114" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D114" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E114" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6">
-      <c r="A115" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B115" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C115" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="D115" s="1">
-        <v>196323.34</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6">
-      <c r="A116" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B116" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C116" s="1">
-        <v>25653898</v>
-      </c>
-      <c r="D116" s="1">
-        <v>1045412.19</v>
-      </c>
-      <c r="E116" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F116" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6">
-      <c r="A117" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B117" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C117" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D117" s="1">
-        <v>11330000</v>
-      </c>
-      <c r="E117" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F117" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6">
-      <c r="A118" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B118" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D118" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E118" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F118" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6">
-      <c r="A119" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D119" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E119" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F119" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6">
-      <c r="A120" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D120" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E120" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F120" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6">
-      <c r="A121" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B121" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C121" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D121" s="1">
-        <v>1909070.4</v>
-      </c>
-      <c r="E121" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F121" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6">
-      <c r="A122" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B122" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C122" s="1">
-        <v>84947615</v>
-      </c>
-      <c r="D122" s="1">
-        <v>39548690.640000001</v>
-      </c>
-      <c r="E122" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F122" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6">
-      <c r="A123" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B123" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C123" s="1">
-        <v>105979279</v>
-      </c>
-      <c r="D123" s="1">
-        <v>27987852.739999998</v>
-      </c>
-      <c r="E123" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F123" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6">
-      <c r="A124" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C124" s="1">
-        <v>105979279</v>
-      </c>
-      <c r="D124" s="1">
-        <v>1031000.99</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F124" s="1" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
upgrade:update snapshot to 20260901 and add .gitignore
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alef.xu/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B3747A0-AE08-B541-99F3-9E44A24EFA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9429CF8-0F2F-9942-957A-803809C69365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3220" yWindow="2140" windowWidth="28100" windowHeight="17360" xr2:uid="{03C76504-C1EF-8B4F-A950-9E551D24283C}"/>
+    <workbookView xWindow="340" yWindow="500" windowWidth="28100" windowHeight="16560" xr2:uid="{A36C5058-2F1C-3B40-B038-45B73BD959AB}"/>
   </bookViews>
   <sheets>
     <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="265" uniqueCount="98">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="364" uniqueCount="110">
   <si>
     <t>coin</t>
   </si>
@@ -75,12 +75,18 @@
     <t>HTX(All)</t>
   </si>
   <si>
+    <t>232059560281012.00</t>
+  </si>
+  <si>
     <t>HTX-ERC20</t>
   </si>
   <si>
     <t>HTX-TRC20</t>
   </si>
   <si>
+    <t>231371738784003.00</t>
+  </si>
+  <si>
     <t>SOL(All)</t>
   </si>
   <si>
@@ -207,6 +213,33 @@
     <t>TK86Qm97uM848dMk8G7xNbJB7zG1uW3h1n</t>
   </si>
   <si>
+    <t>TWN6yGR6VzYmThSy2CmkpEASyvwV4VKRDs</t>
+  </si>
+  <si>
+    <t>htx</t>
+  </si>
+  <si>
+    <t>0x4c1d4b5922317f58967c3759c6bbeb57497e40e81662260ae8fa82496d0c391467a0d0cf7d8bd9039594057c4353c7d7831c247912148a62f9548282372a551700</t>
+  </si>
+  <si>
+    <t>TB5s4duG2LqfnkF1VgX4fWdvtYcmf1WELk</t>
+  </si>
+  <si>
+    <t>0xf0d92874a3a44f7ecaec706de6c481f003baab5373c0cd98c73aa2d911ff029a432e8c42150546d1a72b21cf0326a28077fa01e4c6d91a256b13c225c84b26b901</t>
+  </si>
+  <si>
+    <t>THBF3NdL2qRJc19eDCrC5atW3Tdkcg4oMB</t>
+  </si>
+  <si>
+    <t>0x3ca7a1fcc5306107b4bd37c82359ec2a1c62b32658bb01201f12bf5e9e1b5c54623f440d226165bf4d216cffe5a4e3fce9e636e7514eac5c29af97df12e88fd400</t>
+  </si>
+  <si>
+    <t>TYYu2LkRMmd6mH2gCHAQpP8KRSu7CyoHgV</t>
+  </si>
+  <si>
+    <t>0x543ae6227abac6fcf74c224d67acab8d84ee2271a839856dd2fba29af42da08d14389f172454d67d60dac16d4cfd72cd6c3c4efc2fa3c5531d4c153e24cb413400</t>
+  </si>
+  <si>
     <t>DQhEuTa5UkNcD8YFZK3pvjFfrtMqQpJhSa</t>
   </si>
   <si>
@@ -256,6 +289,9 @@
   </si>
   <si>
     <t>0x68a79a40adfb16777e49206d60f9cd11de0fbaf3acad5be1e30dd955182475f43255dfec5fede4dc97fcf1fbce1583dd05ee419bf3939ca95919aff931eec41d01</t>
+  </si>
+  <si>
+    <t>230974428784003.00</t>
   </si>
   <si>
     <t>TYh6mgoMNZTCsgpYHBz7gttEfrQmDMABub</t>
@@ -326,7 +362,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -929,14 +965,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1313,15 +1352,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD334E2B-7567-3B4F-9978-76C3980BF025}">
-  <dimension ref="A1:F92"/>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4067D0-83EE-2E49-A682-3F955B59A64A}">
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="45.33203125" customWidth="1"/>
-    <col min="3" max="3" width="49.6640625" customWidth="1"/>
-    <col min="4" max="4" width="63.5" customWidth="1"/>
-    <col min="5" max="5" width="22.1640625" customWidth="1"/>
-    <col min="6" max="6" width="127.33203125" customWidth="1"/>
+    <col min="2" max="2" width="59.1640625" customWidth="1"/>
+    <col min="3" max="3" width="83" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="143.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1463,13 +1502,13 @@
       <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="2">
-        <v>232059560281012</v>
+      <c r="C13" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" s="1">
         <v>25876316</v>
@@ -1480,13 +1519,13 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="1">
         <v>85840149</v>
       </c>
-      <c r="C15" s="2">
-        <v>231371738784003</v>
+      <c r="C15" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1502,7 +1541,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>4</v>
@@ -1513,7 +1552,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1">
         <v>443191405</v>
@@ -1535,7 +1574,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>4</v>
@@ -1546,7 +1585,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B21" s="1">
         <v>85840149</v>
@@ -1557,7 +1596,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B22" s="1">
         <v>85840149</v>
@@ -1568,7 +1607,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>4</v>
@@ -1579,7 +1618,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B24" s="1">
         <v>106670116</v>
@@ -1590,7 +1629,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>4</v>
@@ -1601,7 +1640,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B26" s="1">
         <v>443191405</v>
@@ -1623,7 +1662,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>4</v>
@@ -1634,7 +1673,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B29" s="1">
         <v>85840149</v>
@@ -1656,7 +1695,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>4</v>
@@ -1667,7 +1706,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B32" s="1">
         <v>85840149</v>
@@ -1678,7 +1717,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" s="1">
         <v>85840149</v>
@@ -1700,7 +1739,7 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>4</v>
@@ -1711,7 +1750,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1">
         <v>25876316</v>
@@ -1722,7 +1761,7 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>4</v>
@@ -1733,7 +1772,7 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B38" s="1">
         <v>85840149</v>
@@ -1744,7 +1783,7 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1">
         <v>85840149</v>
@@ -1755,7 +1794,7 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B40" s="1">
         <v>25876316</v>
@@ -1780,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>1</v>
@@ -1789,10 +1828,10 @@
         <v>2</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1800,7 +1839,7 @@
         <v>5</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C44" s="1">
         <v>964902</v>
@@ -1809,10 +1848,10 @@
         <v>6132.7</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -1820,7 +1859,7 @@
         <v>5</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C45" s="1">
         <v>964902</v>
@@ -1829,10 +1868,10 @@
         <v>970.8</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1840,7 +1879,7 @@
         <v>5</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C46" s="1">
         <v>964902</v>
@@ -1849,10 +1888,10 @@
         <v>8.3800000000000008</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -1860,7 +1899,7 @@
         <v>5</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C47" s="1">
         <v>964902</v>
@@ -1869,10 +1908,10 @@
         <v>829.68</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1880,7 +1919,7 @@
         <v>5</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C48" s="1">
         <v>964902</v>
@@ -1900,7 +1939,7 @@
         <v>5</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C49" s="1">
         <v>964902</v>
@@ -1909,10 +1948,10 @@
         <v>46.26</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -1920,7 +1959,7 @@
         <v>5</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C50" s="1">
         <v>964902</v>
@@ -1940,7 +1979,7 @@
         <v>6</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C51" s="1">
         <v>443191405</v>
@@ -1960,7 +1999,7 @@
         <v>6</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C52" s="1">
         <v>443191405</v>
@@ -1980,7 +2019,7 @@
         <v>7</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C53" s="1">
         <v>85840149</v>
@@ -1989,10 +2028,10 @@
         <v>10298.93</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2000,7 +2039,7 @@
         <v>7</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C54" s="1">
         <v>85840149</v>
@@ -2017,102 +2056,102 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C55" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D55" s="1">
-        <v>89</v>
+        <v>62</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C56" s="1">
-        <v>6355057</v>
-      </c>
-      <c r="D56" s="1">
-        <v>1189758.8700000001</v>
+        <v>65</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C57" s="1">
-        <v>6355057</v>
-      </c>
-      <c r="D57" s="1">
-        <v>342891003.5</v>
+        <v>67</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C58" s="1">
-        <v>6355057</v>
-      </c>
-      <c r="D58" s="1">
-        <v>66066923.390000001</v>
+        <v>69</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C59" s="1">
-        <v>6355057</v>
+        <v>85840149</v>
       </c>
       <c r="D59" s="1">
-        <v>2866994</v>
+        <v>89</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2120,13 +2159,13 @@
         <v>12</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C60" s="1">
         <v>6355057</v>
       </c>
       <c r="D60" s="1">
-        <v>2647816.5299999998</v>
+        <v>1189758.8700000001</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>4</v>
@@ -2140,13 +2179,13 @@
         <v>12</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C61" s="1">
         <v>6355057</v>
       </c>
       <c r="D61" s="1">
-        <v>1457329.63</v>
+        <v>342891003.5</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>4</v>
@@ -2160,13 +2199,13 @@
         <v>12</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C62" s="1">
         <v>6355057</v>
       </c>
       <c r="D62" s="1">
-        <v>1066964.3</v>
+        <v>66066923.390000001</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>4</v>
@@ -2180,13 +2219,13 @@
         <v>12</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C63" s="1">
         <v>6355057</v>
       </c>
       <c r="D63" s="1">
-        <v>850746.71</v>
+        <v>2866994</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>4</v>
@@ -2200,13 +2239,13 @@
         <v>12</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C64" s="1">
         <v>6355057</v>
       </c>
       <c r="D64" s="1">
-        <v>579364.13</v>
+        <v>2647816.5299999998</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>4</v>
@@ -2220,13 +2259,13 @@
         <v>12</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C65" s="1">
         <v>6355057</v>
       </c>
       <c r="D65" s="1">
-        <v>538350.48</v>
+        <v>1457329.63</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>4</v>
@@ -2240,13 +2279,13 @@
         <v>12</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C66" s="1">
         <v>6355057</v>
       </c>
       <c r="D66" s="1">
-        <v>127419.44</v>
+        <v>1066964.3</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>4</v>
@@ -2260,13 +2299,13 @@
         <v>12</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C67" s="1">
         <v>6355057</v>
       </c>
       <c r="D67" s="1">
-        <v>999998.92</v>
+        <v>850746.71</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>4</v>
@@ -2280,13 +2319,13 @@
         <v>12</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C68" s="1">
         <v>6355057</v>
       </c>
       <c r="D68" s="1">
-        <v>999999.11</v>
+        <v>579364.13</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>4</v>
@@ -2300,13 +2339,13 @@
         <v>12</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C69" s="1">
         <v>6355057</v>
       </c>
       <c r="D69" s="1">
-        <v>477914.18</v>
+        <v>538350.48</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>4</v>
@@ -2317,16 +2356,16 @@
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="C70" s="1">
-        <v>25876316</v>
+        <v>6355057</v>
       </c>
       <c r="D70" s="1">
-        <v>29213.08</v>
+        <v>127419.44</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>4</v>
@@ -2337,56 +2376,56 @@
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C71" s="1">
-        <v>25876316</v>
-      </c>
-      <c r="D71" s="2">
-        <v>386057650000</v>
+        <v>6355057</v>
+      </c>
+      <c r="D71" s="1">
+        <v>999998.92</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>76</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="C72" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D72" s="2">
-        <v>230974428784003</v>
+        <v>6355057</v>
+      </c>
+      <c r="D72" s="1">
+        <v>999999.11</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>58</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C73" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D73" s="2">
-        <v>397310000000</v>
+        <v>6355057</v>
+      </c>
+      <c r="D73" s="1">
+        <v>477914.18</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>4</v>
@@ -2397,16 +2436,16 @@
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="C74" s="1">
-        <v>443191405</v>
+        <v>25876316</v>
       </c>
       <c r="D74" s="1">
-        <v>399536.39</v>
+        <v>29213.08</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>4</v>
@@ -2417,336 +2456,336 @@
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="C75" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D75" s="1">
-        <v>1082089494.28</v>
+        <v>25876316</v>
+      </c>
+      <c r="D75" s="2">
+        <v>386057650000</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="C76" s="1">
         <v>85840149</v>
       </c>
-      <c r="D76" s="1">
-        <v>1705110564.0899999</v>
+      <c r="D76" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="C77" s="1">
         <v>85840149</v>
       </c>
-      <c r="D77" s="1">
-        <v>755759959.02999997</v>
+      <c r="D77" s="2">
+        <v>397310000000</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C78" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D78" s="1">
-        <v>1071286648.08</v>
+        <v>62</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C79" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D79" s="1">
-        <v>1070397075.17</v>
+        <v>65</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C80" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D80" s="1">
-        <v>1144452002.4400001</v>
+        <v>67</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C81" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D81" s="1">
-        <v>1632640336.6900001</v>
+        <v>69</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="C82" s="1">
-        <v>85840149</v>
+        <v>443191405</v>
       </c>
       <c r="D82" s="1">
-        <v>922473805.94000006</v>
+        <v>399536.39</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>92</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="C83" s="1">
         <v>85840149</v>
       </c>
       <c r="D83" s="1">
-        <v>14984999</v>
+        <v>1082089494.28</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>4</v>
+        <v>90</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="C84" s="1">
-        <v>443191405</v>
+        <v>85840149</v>
       </c>
       <c r="D84" s="1">
-        <v>972000</v>
+        <v>1705110564.0899999</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>4</v>
+        <v>92</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="1" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="C85" s="1">
         <v>85840149</v>
       </c>
       <c r="D85" s="1">
-        <v>2681000</v>
+        <v>755759959.02999997</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>4</v>
+        <v>94</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="1" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>57</v>
+        <v>95</v>
       </c>
       <c r="C86" s="1">
         <v>85840149</v>
       </c>
       <c r="D86" s="1">
-        <v>76466743.670000002</v>
+        <v>1071286648.08</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>58</v>
+        <v>96</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="C87" s="1">
-        <v>25876316</v>
+        <v>85840149</v>
       </c>
       <c r="D87" s="1">
-        <v>44975772</v>
+        <v>1070397075.17</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C88" s="1">
-        <v>25876316</v>
+        <v>85840149</v>
       </c>
       <c r="D88" s="1">
-        <v>360949.9</v>
+        <v>1144452002.4400001</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="1" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="C89" s="1">
         <v>85840149</v>
       </c>
       <c r="D89" s="1">
-        <v>1909070.4</v>
+        <v>1632640336.6900001</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>57</v>
+        <v>103</v>
       </c>
       <c r="C90" s="1">
         <v>85840149</v>
       </c>
       <c r="D90" s="1">
-        <v>39548690.640000001</v>
+        <v>922473805.94000006</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>58</v>
+        <v>104</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="C91" s="1">
-        <v>106670116</v>
+        <v>85840149</v>
       </c>
       <c r="D91" s="1">
-        <v>26487852.739999998</v>
+        <v>14984999</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>4</v>
@@ -2757,26 +2796,346 @@
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C92" s="1">
+        <v>62</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C96" s="1">
+        <v>443191405</v>
+      </c>
+      <c r="D96" s="1">
+        <v>972000</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C97" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D97" s="1">
+        <v>2681000</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
+      <c r="A98" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
+      <c r="A101" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
+      <c r="A102" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C102" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D102" s="1">
+        <v>76466743.670000002</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
+      <c r="A103" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C103" s="1">
+        <v>25876316</v>
+      </c>
+      <c r="D103" s="1">
+        <v>44975772</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C104" s="1">
+        <v>25876316</v>
+      </c>
+      <c r="D104" s="1">
+        <v>360949.9</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C105" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D105" s="1">
+        <v>1909070.4</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6">
+      <c r="A106" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C106" s="1">
+        <v>85840149</v>
+      </c>
+      <c r="D106" s="1">
+        <v>39548690.640000001</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
+      <c r="A107" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C107" s="1">
         <v>106670116</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D107" s="1">
+        <v>26487852.739999998</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
+      <c r="A108" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C108" s="1">
+        <v>106670116</v>
+      </c>
+      <c r="D108" s="1">
         <v>894000.99</v>
       </c>
-      <c r="E92" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F92" s="1" t="s">
+      <c r="E108" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F108" s="1" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>